<commit_message>
feat: Implement new `StatsScraper` with robust hierarchical data fetching and validation, and add new model training metrics.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-15.xlsx
+++ b/results/nba_predictions_2025-12-15.xlsx
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>59.38</v>
+        <v>59.09</v>
       </c>
       <c r="E2" t="n">
-        <v>40.62</v>
+        <v>40.91</v>
       </c>
       <c r="F2" t="n">
         <v>59.61</v>
@@ -608,13 +608,13 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>59.4</v>
+        <v>59.1</v>
       </c>
       <c r="S2" t="n">
-        <v>40.6</v>
+        <v>40.9</v>
       </c>
       <c r="T2" t="n">
-        <v>233.3</v>
+        <v>225.3</v>
       </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="3">
@@ -643,16 +643,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>57.81</v>
+        <v>56.25</v>
       </c>
       <c r="E3" t="n">
-        <v>42.19</v>
+        <v>43.75</v>
       </c>
       <c r="F3" t="n">
-        <v>59.21</v>
+        <v>59.12</v>
       </c>
       <c r="G3" t="n">
-        <v>40.79</v>
+        <v>40.88</v>
       </c>
       <c r="H3" t="n">
         <v>-0.11</v>
@@ -689,13 +689,13 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>57.8</v>
+        <v>56.2</v>
       </c>
       <c r="S3" t="n">
-        <v>42.2</v>
+        <v>43.8</v>
       </c>
       <c r="T3" t="n">
-        <v>220.6</v>
+        <v>223.3</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -704,7 +704,7 @@
       </c>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="n">
-        <v>4.7</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="4">
@@ -724,16 +724,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>57.81</v>
+        <v>46.67</v>
       </c>
       <c r="E4" t="n">
-        <v>42.19</v>
+        <v>53.33</v>
       </c>
       <c r="F4" t="n">
-        <v>56.54</v>
+        <v>56.57</v>
       </c>
       <c r="G4" t="n">
-        <v>43.46</v>
+        <v>43.43</v>
       </c>
       <c r="H4" t="n">
         <v>-0.62</v>
@@ -755,7 +755,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -770,13 +770,13 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>57.8</v>
+        <v>46.7</v>
       </c>
       <c r="S4" t="n">
-        <v>42.2</v>
+        <v>53.3</v>
       </c>
       <c r="T4" t="n">
-        <v>211.5</v>
+        <v>236</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="W4" t="n">
-        <v>4.7</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="5">
@@ -809,10 +809,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>50</v>
+        <v>33.33</v>
       </c>
       <c r="E5" t="n">
-        <v>50</v>
+        <v>66.67</v>
       </c>
       <c r="F5" t="n">
         <v>56.85</v>
@@ -840,7 +840,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -855,13 +855,13 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>50</v>
+        <v>33.3</v>
       </c>
       <c r="S5" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="T5" t="n">
-        <v>229.6</v>
+        <v>238.7</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
         </is>
       </c>
       <c r="W5" t="n">
-        <v>0</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="6">
@@ -894,16 +894,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>57.81</v>
+        <v>33.33</v>
       </c>
       <c r="E6" t="n">
-        <v>42.19</v>
+        <v>66.67</v>
       </c>
       <c r="F6" t="n">
-        <v>56.3</v>
+        <v>56.19</v>
       </c>
       <c r="G6" t="n">
-        <v>43.7</v>
+        <v>43.81</v>
       </c>
       <c r="H6" t="n">
         <v>0.03</v>
@@ -925,7 +925,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -940,13 +940,13 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>57.8</v>
+        <v>33.3</v>
       </c>
       <c r="S6" t="n">
-        <v>42.2</v>
+        <v>66.7</v>
       </c>
       <c r="T6" t="n">
-        <v>208</v>
+        <v>236</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -959,7 +959,7 @@
         </is>
       </c>
       <c r="W6" t="n">
-        <v>4.7</v>
+        <v>-10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Implement odds fetching with multiple providers, custom exceptions, Redis-based quota management, and Playwright support in Docker.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-15.xlsx
+++ b/results/nba_predictions_2025-12-15.xlsx
@@ -562,16 +562,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>59.09</v>
+        <v>59.38</v>
       </c>
       <c r="E2" t="n">
-        <v>40.91</v>
+        <v>40.62</v>
       </c>
       <c r="F2" t="n">
-        <v>59.61</v>
+        <v>59.52</v>
       </c>
       <c r="G2" t="n">
-        <v>40.39</v>
+        <v>40.48</v>
       </c>
       <c r="H2" t="n">
         <v>0.32</v>
@@ -608,13 +608,13 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>59.1</v>
+        <v>59.4</v>
       </c>
       <c r="S2" t="n">
-        <v>40.9</v>
+        <v>40.6</v>
       </c>
       <c r="T2" t="n">
-        <v>225.3</v>
+        <v>233.3</v>
       </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="3">
@@ -643,16 +643,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>56.25</v>
+        <v>57.81</v>
       </c>
       <c r="E3" t="n">
-        <v>43.75</v>
+        <v>42.19</v>
       </c>
       <c r="F3" t="n">
-        <v>59.12</v>
+        <v>59.13</v>
       </c>
       <c r="G3" t="n">
-        <v>40.88</v>
+        <v>40.87</v>
       </c>
       <c r="H3" t="n">
         <v>-0.11</v>
@@ -689,13 +689,13 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>56.2</v>
+        <v>57.8</v>
       </c>
       <c r="S3" t="n">
-        <v>43.8</v>
+        <v>42.2</v>
       </c>
       <c r="T3" t="n">
-        <v>223.3</v>
+        <v>220.6</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -704,7 +704,7 @@
       </c>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="n">
-        <v>3.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="4">
@@ -724,16 +724,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>46.67</v>
+        <v>57.81</v>
       </c>
       <c r="E4" t="n">
-        <v>53.33</v>
+        <v>42.19</v>
       </c>
       <c r="F4" t="n">
-        <v>56.57</v>
+        <v>56.53</v>
       </c>
       <c r="G4" t="n">
-        <v>43.43</v>
+        <v>43.47</v>
       </c>
       <c r="H4" t="n">
         <v>-0.62</v>
@@ -755,7 +755,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -770,13 +770,13 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>46.7</v>
+        <v>57.8</v>
       </c>
       <c r="S4" t="n">
-        <v>53.3</v>
+        <v>42.2</v>
       </c>
       <c r="T4" t="n">
-        <v>236</v>
+        <v>211.5</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="W4" t="n">
-        <v>-2</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="5">
@@ -809,16 +809,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>33.33</v>
+        <v>50</v>
       </c>
       <c r="E5" t="n">
-        <v>66.67</v>
+        <v>50</v>
       </c>
       <c r="F5" t="n">
-        <v>56.85</v>
+        <v>56.86</v>
       </c>
       <c r="G5" t="n">
-        <v>43.15</v>
+        <v>43.14</v>
       </c>
       <c r="H5" t="n">
         <v>-0.06</v>
@@ -840,7 +840,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -855,13 +855,13 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="S5" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
       <c r="T5" t="n">
-        <v>238.7</v>
+        <v>229.6</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
         </is>
       </c>
       <c r="W5" t="n">
-        <v>-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -894,16 +894,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>33.33</v>
+        <v>57.81</v>
       </c>
       <c r="E6" t="n">
-        <v>66.67</v>
+        <v>42.19</v>
       </c>
       <c r="F6" t="n">
-        <v>56.19</v>
+        <v>56.29</v>
       </c>
       <c r="G6" t="n">
-        <v>43.81</v>
+        <v>43.71</v>
       </c>
       <c r="H6" t="n">
         <v>0.03</v>
@@ -925,7 +925,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -940,13 +940,13 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>33.3</v>
+        <v>57.8</v>
       </c>
       <c r="S6" t="n">
-        <v>66.7</v>
+        <v>42.2</v>
       </c>
       <c r="T6" t="n">
-        <v>236</v>
+        <v>208</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -959,7 +959,7 @@
         </is>
       </c>
       <c r="W6" t="n">
-        <v>-10</v>
+        <v>4.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
git add -A && git commit -m "v26.0: Odds Module Refactoring - Multi-Provider Architecture"
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-15.xlsx
+++ b/results/nba_predictions_2025-12-15.xlsx
@@ -568,10 +568,10 @@
         <v>40.62</v>
       </c>
       <c r="F2" t="n">
-        <v>59.52</v>
+        <v>59.53</v>
       </c>
       <c r="G2" t="n">
-        <v>40.48</v>
+        <v>40.47</v>
       </c>
       <c r="H2" t="n">
         <v>0.32</v>
@@ -649,10 +649,10 @@
         <v>42.19</v>
       </c>
       <c r="F3" t="n">
-        <v>59.13</v>
+        <v>59.1</v>
       </c>
       <c r="G3" t="n">
-        <v>40.87</v>
+        <v>40.9</v>
       </c>
       <c r="H3" t="n">
         <v>-0.11</v>
@@ -730,10 +730,10 @@
         <v>42.19</v>
       </c>
       <c r="F4" t="n">
-        <v>56.53</v>
+        <v>56.56</v>
       </c>
       <c r="G4" t="n">
-        <v>43.47</v>
+        <v>43.44</v>
       </c>
       <c r="H4" t="n">
         <v>-0.62</v>
@@ -900,10 +900,10 @@
         <v>42.19</v>
       </c>
       <c r="F6" t="n">
-        <v>56.29</v>
+        <v>56.34</v>
       </c>
       <c r="G6" t="n">
-        <v>43.71</v>
+        <v>43.66</v>
       </c>
       <c r="H6" t="n">
         <v>0.03</v>

</xml_diff>

<commit_message>
feat: Introduce V22.0 non-linear injury impact modeling, new feature engineering, and ensemble blending modules.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-15.xlsx
+++ b/results/nba_predictions_2025-12-15.xlsx
@@ -568,10 +568,10 @@
         <v>40.62</v>
       </c>
       <c r="F2" t="n">
-        <v>59.53</v>
+        <v>59.54</v>
       </c>
       <c r="G2" t="n">
-        <v>40.47</v>
+        <v>40.46</v>
       </c>
       <c r="H2" t="n">
         <v>0.32</v>
@@ -649,10 +649,10 @@
         <v>42.19</v>
       </c>
       <c r="F3" t="n">
-        <v>59.1</v>
+        <v>59.23</v>
       </c>
       <c r="G3" t="n">
-        <v>40.9</v>
+        <v>40.77</v>
       </c>
       <c r="H3" t="n">
         <v>-0.11</v>
@@ -730,10 +730,10 @@
         <v>42.19</v>
       </c>
       <c r="F4" t="n">
-        <v>56.56</v>
+        <v>56.62</v>
       </c>
       <c r="G4" t="n">
-        <v>43.44</v>
+        <v>43.38</v>
       </c>
       <c r="H4" t="n">
         <v>-0.62</v>
@@ -815,10 +815,10 @@
         <v>50</v>
       </c>
       <c r="F5" t="n">
-        <v>56.86</v>
+        <v>56.81</v>
       </c>
       <c r="G5" t="n">
-        <v>43.14</v>
+        <v>43.19</v>
       </c>
       <c r="H5" t="n">
         <v>-0.06</v>
@@ -900,10 +900,10 @@
         <v>42.19</v>
       </c>
       <c r="F6" t="n">
-        <v>56.34</v>
+        <v>56.28</v>
       </c>
       <c r="G6" t="n">
-        <v>43.66</v>
+        <v>43.72</v>
       </c>
       <c r="H6" t="n">
         <v>0.03</v>

</xml_diff>